<commit_message>
give the pi-score count a permutation null it never had
</commit_message>
<xml_diff>
--- a/04_Features/modules/c_data/module_contrasts.xlsx
+++ b/04_Features/modules/c_data/module_contrasts.xlsx
@@ -459,16 +459,16 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>0.17425092658077</v>
+        <v>0.163440551488145</v>
       </c>
       <c r="D2" t="n">
-        <v>2.3274237199715</v>
+        <v>2.18610964342696</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0204071679468525</v>
+        <v>0.029347354796083</v>
       </c>
       <c r="F2" t="n">
-        <v>0.224478847415378</v>
+        <v>0.236962350301216</v>
       </c>
     </row>
     <row r="3">
@@ -479,16 +479,16 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00461843191688611</v>
+        <v>0.00984263494844101</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0616871783889867</v>
+        <v>0.131650798908855</v>
       </c>
       <c r="E3" t="n">
-        <v>0.950840679229933</v>
+        <v>0.895322222176802</v>
       </c>
       <c r="F3" t="n">
-        <v>0.960146595097477</v>
+        <v>0.895322222176802</v>
       </c>
     </row>
     <row r="4">
@@ -499,16 +499,16 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.145404468260077</v>
+        <v>0.015351710135656</v>
       </c>
       <c r="D4" t="n">
-        <v>1.94212917577503</v>
+        <v>0.205337789582088</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0527756256599646</v>
+        <v>0.837405617197178</v>
       </c>
       <c r="F4" t="n">
-        <v>0.255336764787751</v>
+        <v>0.895322222176802</v>
       </c>
     </row>
     <row r="5">
@@ -519,16 +519,16 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.119870424819134</v>
+        <v>-0.127629100798965</v>
       </c>
       <c r="D5" t="n">
-        <v>-1.60107768447242</v>
+        <v>-1.70711127378182</v>
       </c>
       <c r="E5" t="n">
-        <v>0.110095794873296</v>
+        <v>0.0885249459641226</v>
       </c>
       <c r="F5" t="n">
-        <v>0.255336764787751</v>
+        <v>0.265231963101765</v>
       </c>
     </row>
     <row r="6">
@@ -539,16 +539,16 @@
         <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0695662929791277</v>
+        <v>0.0100615119654476</v>
       </c>
       <c r="D6" t="n">
-        <v>0.929178648097797</v>
+        <v>0.1345784025742</v>
       </c>
       <c r="E6" t="n">
-        <v>0.35331903045467</v>
+        <v>0.893008333416084</v>
       </c>
       <c r="F6" t="n">
-        <v>0.485813666875172</v>
+        <v>0.895322222176802</v>
       </c>
     </row>
     <row r="7">
@@ -559,16 +559,16 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.102069989661726</v>
+        <v>-0.102025442833883</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.3633219615956</v>
+        <v>-1.36464789443785</v>
       </c>
       <c r="E7" t="n">
-        <v>0.17349609883131</v>
+        <v>0.173079085736162</v>
       </c>
       <c r="F7" t="n">
-        <v>0.318076181190734</v>
+        <v>0.317311657182965</v>
       </c>
     </row>
     <row r="8">
@@ -579,16 +579,16 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0182622226962919</v>
+        <v>0.124553760281588</v>
       </c>
       <c r="D8" t="n">
-        <v>0.243923697375864</v>
+        <v>1.66597685823656</v>
       </c>
       <c r="E8" t="n">
-        <v>0.807406522566315</v>
+        <v>0.09644798658246</v>
       </c>
       <c r="F8" t="n">
-        <v>0.960146595097477</v>
+        <v>0.265231963101765</v>
       </c>
     </row>
     <row r="9">
@@ -599,16 +599,16 @@
         <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>0.125170010431124</v>
+        <v>0.0697153223915064</v>
       </c>
       <c r="D9" t="n">
-        <v>1.67186285331712</v>
+        <v>0.932481793453485</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0952805350550737</v>
+        <v>0.351612083078058</v>
       </c>
       <c r="F9" t="n">
-        <v>0.255336764787751</v>
+        <v>0.48346661423233</v>
       </c>
     </row>
     <row r="10">
@@ -619,16 +619,16 @@
         <v>15</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0872939501086421</v>
+        <v>0.079943899575923</v>
       </c>
       <c r="D10" t="n">
-        <v>1.16596229402939</v>
+        <v>1.06929478764491</v>
       </c>
       <c r="E10" t="n">
-        <v>0.244277496561677</v>
+        <v>0.285538134588101</v>
       </c>
       <c r="F10" t="n">
-        <v>0.383864637454063</v>
+        <v>0.448702782924159</v>
       </c>
     </row>
     <row r="11">
@@ -639,16 +639,16 @@
         <v>16</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.117895785723807</v>
+        <v>-0.115888431052053</v>
       </c>
       <c r="D11" t="n">
-        <v>-1.57470295029437</v>
+        <v>-1.55007318794376</v>
       </c>
       <c r="E11" t="n">
-        <v>0.116062165812614</v>
+        <v>0.121861319342874</v>
       </c>
       <c r="F11" t="n">
-        <v>0.255336764787751</v>
+        <v>0.268094902554322</v>
       </c>
     </row>
     <row r="12">
@@ -659,16 +659,16 @@
         <v>17</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0037433413698872</v>
+        <v>0.151688130833931</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0499988244951321</v>
+        <v>2.02891438256998</v>
       </c>
       <c r="E12" t="n">
-        <v>0.960146595097477</v>
+        <v>0.0430840636911303</v>
       </c>
       <c r="F12" t="n">
-        <v>0.960146595097477</v>
+        <v>0.236962350301216</v>
       </c>
     </row>
     <row r="13">
@@ -679,16 +679,16 @@
         <v>7</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0887187279761334</v>
+        <v>0.0599806462511723</v>
       </c>
       <c r="D13" t="n">
-        <v>1.27700058066186</v>
+        <v>0.865771988156715</v>
       </c>
       <c r="E13" t="n">
-        <v>0.202292779264323</v>
+        <v>0.387099121710436</v>
       </c>
       <c r="F13" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="14">
@@ -699,16 +699,16 @@
         <v>8</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00664479106411173</v>
+        <v>0.0324948861199908</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0956438650645454</v>
+        <v>0.469037329861724</v>
       </c>
       <c r="E14" t="n">
-        <v>0.923848085773366</v>
+        <v>0.639281220645106</v>
       </c>
       <c r="F14" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="15">
@@ -719,16 +719,16 @@
         <v>9</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0113712482267952</v>
+        <v>0.00640984062376629</v>
       </c>
       <c r="D15" t="n">
-        <v>0.163675594992457</v>
+        <v>0.0925208514320959</v>
       </c>
       <c r="E15" t="n">
-        <v>0.870063610774027</v>
+        <v>0.926327414679895</v>
       </c>
       <c r="F15" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="16">
@@ -739,16 +739,16 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.00433049874317533</v>
+        <v>-0.0201423238526641</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0623323793717828</v>
+        <v>-0.290738110673101</v>
       </c>
       <c r="E16" t="n">
-        <v>0.950327173765851</v>
+        <v>0.771392121562186</v>
       </c>
       <c r="F16" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="17">
@@ -759,16 +759,16 @@
         <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0154778749012223</v>
+        <v>0.017186749613667</v>
       </c>
       <c r="D17" t="n">
-        <v>0.222785602173982</v>
+        <v>0.248076793315399</v>
       </c>
       <c r="E17" t="n">
-        <v>0.823808406517541</v>
+        <v>0.804193690430241</v>
       </c>
       <c r="F17" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="18">
@@ -779,16 +779,16 @@
         <v>12</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.00666295405271881</v>
+        <v>-0.00701978614699099</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0959052996852496</v>
+        <v>-0.101324920432923</v>
       </c>
       <c r="E18" t="n">
-        <v>0.92364056880673</v>
+        <v>0.919339873221008</v>
       </c>
       <c r="F18" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="19">
@@ -799,16 +799,16 @@
         <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0133069405380289</v>
+        <v>0.020024990292107</v>
       </c>
       <c r="D19" t="n">
-        <v>0.191537583794789</v>
+        <v>0.289044495876493</v>
       </c>
       <c r="E19" t="n">
-        <v>0.848195058698829</v>
+        <v>0.772686950588943</v>
       </c>
       <c r="F19" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="20">
@@ -819,16 +819,16 @@
         <v>14</v>
       </c>
       <c r="C20" t="n">
-        <v>0.023496990295322</v>
+        <v>0.0115077229662646</v>
       </c>
       <c r="D20" t="n">
-        <v>0.338211231556479</v>
+        <v>0.166104648988587</v>
       </c>
       <c r="E20" t="n">
-        <v>0.735369463411301</v>
+        <v>0.86815284917739</v>
       </c>
       <c r="F20" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="21">
@@ -839,16 +839,16 @@
         <v>15</v>
       </c>
       <c r="C21" t="n">
-        <v>0.00479271567000719</v>
+        <v>0.00560771240019357</v>
       </c>
       <c r="D21" t="n">
-        <v>0.068985442343051</v>
+        <v>0.0809427809996588</v>
       </c>
       <c r="E21" t="n">
-        <v>0.94503334984807</v>
+        <v>0.935525204626051</v>
       </c>
       <c r="F21" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="22">
@@ -859,16 +859,16 @@
         <v>16</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.0207367056611498</v>
+        <v>-0.0200855892274226</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.298480216910076</v>
+        <v>-0.289919192365902</v>
       </c>
       <c r="E22" t="n">
-        <v>0.765481190564536</v>
+        <v>0.772018134318984</v>
       </c>
       <c r="F22" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="23">
@@ -879,16 +879,16 @@
         <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0177842856521897</v>
+        <v>0.0199833944208887</v>
       </c>
       <c r="D23" t="n">
-        <v>0.25598364204018</v>
+        <v>0.288444093207056</v>
       </c>
       <c r="E23" t="n">
-        <v>0.798086166305484</v>
+        <v>0.773146132606368</v>
       </c>
       <c r="F23" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
     <row r="24">
@@ -899,16 +899,16 @@
         <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.134267572014771</v>
+        <v>-0.122966682906332</v>
       </c>
       <c r="D24" t="n">
-        <v>-1.80780236586594</v>
+        <v>-1.6602897009255</v>
       </c>
       <c r="E24" t="n">
-        <v>0.071337504857376</v>
+        <v>0.0975868817644897</v>
       </c>
       <c r="F24" t="n">
-        <v>0.156942510686227</v>
+        <v>0.214691139881877</v>
       </c>
     </row>
     <row r="25">
@@ -919,16 +919,16 @@
         <v>8</v>
       </c>
       <c r="C25" t="n">
-        <v>0.138659313379964</v>
+        <v>0.136019740501266</v>
       </c>
       <c r="D25" t="n">
-        <v>1.8669335493016</v>
+        <v>1.83653139971935</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0625927404040017</v>
+        <v>0.0669708208120773</v>
       </c>
       <c r="F25" t="n">
-        <v>0.156942510686227</v>
+        <v>0.184169757233212</v>
       </c>
     </row>
     <row r="26">
@@ -939,16 +939,16 @@
         <v>9</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.201537382986135</v>
+        <v>-0.184370431711183</v>
       </c>
       <c r="D26" t="n">
-        <v>-2.71353501300137</v>
+        <v>-2.48935989562669</v>
       </c>
       <c r="E26" t="n">
-        <v>0.00692506393730139</v>
+        <v>0.0131752591918906</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0761757033103153</v>
+        <v>0.0697935914744919</v>
       </c>
     </row>
     <row r="27">
@@ -959,16 +959,16 @@
         <v>10</v>
       </c>
       <c r="C27" t="n">
-        <v>0.0860009796394341</v>
+        <v>0.076664332400634</v>
       </c>
       <c r="D27" t="n">
-        <v>1.15793241901963</v>
+        <v>1.03511779373653</v>
       </c>
       <c r="E27" t="n">
-        <v>0.24753585628794</v>
+        <v>0.301197033966177</v>
       </c>
       <c r="F27" t="n">
-        <v>0.45381573652789</v>
+        <v>0.473309624803992</v>
       </c>
     </row>
     <row r="28">
@@ -979,16 +979,16 @@
         <v>11</v>
       </c>
       <c r="C28" t="n">
-        <v>-0.0756058703989498</v>
+        <v>0.174327763077681</v>
       </c>
       <c r="D28" t="n">
-        <v>-1.01797082742762</v>
+        <v>2.35376431064444</v>
       </c>
       <c r="E28" t="n">
-        <v>0.309265558677127</v>
+        <v>0.0190346158566796</v>
       </c>
       <c r="F28" t="n">
-        <v>0.485988735064057</v>
+        <v>0.0697935914744919</v>
       </c>
     </row>
     <row r="29">
@@ -999,16 +999,16 @@
         <v>12</v>
       </c>
       <c r="C29" t="n">
-        <v>0.0580905756380288</v>
+        <v>0.0609189079196564</v>
       </c>
       <c r="D29" t="n">
-        <v>0.782141797137653</v>
+        <v>0.822523898507362</v>
       </c>
       <c r="E29" t="n">
-        <v>0.434562721128356</v>
+        <v>0.411235730263329</v>
       </c>
       <c r="F29" t="n">
-        <v>0.531132214712436</v>
+        <v>0.502621448099624</v>
       </c>
     </row>
     <row r="30">
@@ -1019,16 +1019,16 @@
         <v>13</v>
       </c>
       <c r="C30" t="n">
-        <v>0.172240437979974</v>
+        <v>-0.00630213084190683</v>
       </c>
       <c r="D30" t="n">
-        <v>2.31907575750104</v>
+        <v>-0.0850910399744067</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0208598776799607</v>
+        <v>0.932228708918963</v>
       </c>
       <c r="F30" t="n">
-        <v>0.076486218159856</v>
+        <v>0.932228708918963</v>
       </c>
     </row>
     <row r="31">
@@ -1039,16 +1039,16 @@
         <v>14</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.012242707258276</v>
+        <v>-0.0801913374957558</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.164837978478382</v>
+        <v>-1.08273923147998</v>
       </c>
       <c r="E31" t="n">
-        <v>0.869149151821834</v>
+        <v>0.279532375115614</v>
       </c>
       <c r="F31" t="n">
-        <v>0.869149151821834</v>
+        <v>0.473309624803992</v>
       </c>
     </row>
     <row r="32">
@@ -1059,16 +1059,16 @@
         <v>15</v>
       </c>
       <c r="C32" t="n">
-        <v>-0.032247605111012</v>
+        <v>-0.013865770340698</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.434187465658383</v>
+        <v>-0.187214903646668</v>
       </c>
       <c r="E32" t="n">
-        <v>0.664370598154253</v>
+        <v>0.85158064816306</v>
       </c>
       <c r="F32" t="n">
-        <v>0.730807657969679</v>
+        <v>0.932228708918963</v>
       </c>
     </row>
     <row r="33">
@@ -1079,16 +1079,16 @@
         <v>16</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0663536601440665</v>
+        <v>0.0634319103425053</v>
       </c>
       <c r="D33" t="n">
-        <v>0.893397430163637</v>
+        <v>0.85645432537132</v>
       </c>
       <c r="E33" t="n">
-        <v>0.372145270872292</v>
+        <v>0.392224659362268</v>
       </c>
       <c r="F33" t="n">
-        <v>0.511699747449401</v>
+        <v>0.502621448099624</v>
       </c>
     </row>
     <row r="34">
@@ -1099,16 +1099,16 @@
         <v>17</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.182328952689138</v>
+        <v>-0.188846736971503</v>
       </c>
       <c r="D34" t="n">
-        <v>-2.45490930603124</v>
+        <v>-2.54979873439385</v>
       </c>
       <c r="E34" t="n">
-        <v>0.0144880606336468</v>
+        <v>0.0111252882346163</v>
       </c>
       <c r="F34" t="n">
-        <v>0.076486218159856</v>
+        <v>0.0697935914744919</v>
       </c>
     </row>
     <row r="35">
@@ -1119,16 +1119,16 @@
         <v>7</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.0229610877851472</v>
+        <v>-0.0022894138023219</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.330497552243409</v>
+        <v>-0.033045831667926</v>
       </c>
       <c r="E35" t="n">
-        <v>0.741185386719181</v>
+        <v>0.973653408327096</v>
       </c>
       <c r="F35" t="n">
-        <v>0.815303925391099</v>
+        <v>0.973653408327096</v>
       </c>
     </row>
     <row r="36">
@@ -1139,16 +1139,16 @@
         <v>8</v>
       </c>
       <c r="C36" t="n">
-        <v>0.171674155243678</v>
+        <v>0.0923161271859973</v>
       </c>
       <c r="D36" t="n">
-        <v>2.47104530161644</v>
+        <v>1.33250843343801</v>
       </c>
       <c r="E36" t="n">
-        <v>0.0138594053081593</v>
+        <v>0.183400504194503</v>
       </c>
       <c r="F36" t="n">
-        <v>0.152453458389753</v>
+        <v>0.615570301973216</v>
       </c>
     </row>
     <row r="37">
@@ -1159,16 +1159,16 @@
         <v>9</v>
       </c>
       <c r="C37" t="n">
-        <v>0.00616101253664516</v>
+        <v>-0.100111689545185</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0886804484942274</v>
+        <v>-1.44503105438895</v>
       </c>
       <c r="E37" t="n">
-        <v>0.929377253711649</v>
+        <v>0.149179187303412</v>
       </c>
       <c r="F37" t="n">
-        <v>0.929377253711649</v>
+        <v>0.615570301973216</v>
       </c>
     </row>
     <row r="38">
@@ -1179,16 +1179,16 @@
         <v>10</v>
       </c>
       <c r="C38" t="n">
-        <v>-0.0877014718973078</v>
+        <v>-0.0749696021627394</v>
       </c>
       <c r="D38" t="n">
-        <v>-1.26235838917675</v>
+        <v>-1.08212541165283</v>
       </c>
       <c r="E38" t="n">
-        <v>0.207505651047244</v>
+        <v>0.279804682715098</v>
       </c>
       <c r="F38" t="n">
-        <v>0.540898714652634</v>
+        <v>0.615570301973216</v>
       </c>
     </row>
     <row r="39">
@@ -1199,16 +1199,16 @@
         <v>11</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.0435137770911641</v>
+        <v>0.0386932087352775</v>
       </c>
       <c r="D39" t="n">
-        <v>-0.626329072562398</v>
+        <v>0.558505090369032</v>
       </c>
       <c r="E39" t="n">
-        <v>0.531432234719305</v>
+        <v>0.576790909497371</v>
       </c>
       <c r="F39" t="n">
-        <v>0.751880675854233</v>
+        <v>0.728755774886901</v>
       </c>
     </row>
     <row r="40">
@@ -1219,16 +1219,16 @@
         <v>12</v>
       </c>
       <c r="C40" t="n">
-        <v>0.0390834897963618</v>
+        <v>0.0411641619392544</v>
       </c>
       <c r="D40" t="n">
-        <v>0.562560355663264</v>
+        <v>0.594171296082971</v>
       </c>
       <c r="E40" t="n">
-        <v>0.574028137538539</v>
+        <v>0.552710741564234</v>
       </c>
       <c r="F40" t="n">
-        <v>0.751880675854233</v>
+        <v>0.728755774886901</v>
       </c>
     </row>
     <row r="41">
@@ -1239,16 +1239,16 @@
         <v>13</v>
       </c>
       <c r="C41" t="n">
-        <v>0.034950254340995</v>
+        <v>0.083296048864987</v>
       </c>
       <c r="D41" t="n">
-        <v>0.503067346724548</v>
+        <v>1.20231091758251</v>
       </c>
       <c r="E41" t="n">
-        <v>0.615175098426191</v>
+        <v>0.229906291317126</v>
       </c>
       <c r="F41" t="n">
-        <v>0.751880675854233</v>
+        <v>0.615570301973216</v>
       </c>
     </row>
     <row r="42">
@@ -1259,16 +1259,16 @@
         <v>14</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0807323044692387</v>
+        <v>-0.0367315190075245</v>
       </c>
       <c r="D42" t="n">
-        <v>1.16204551211692</v>
+        <v>-0.530189689954184</v>
       </c>
       <c r="E42" t="n">
-        <v>0.245863052114834</v>
+        <v>0.596254724907464</v>
       </c>
       <c r="F42" t="n">
-        <v>0.540898714652634</v>
+        <v>0.728755774886901</v>
       </c>
     </row>
     <row r="43">
@@ -1279,16 +1279,16 @@
         <v>15</v>
       </c>
       <c r="C43" t="n">
-        <v>0.086693100125935</v>
+        <v>0.105570069561678</v>
       </c>
       <c r="D43" t="n">
-        <v>1.24784407673178</v>
+        <v>1.52381834352894</v>
       </c>
       <c r="E43" t="n">
-        <v>0.212768837336716</v>
+        <v>0.128290895611022</v>
       </c>
       <c r="F43" t="n">
-        <v>0.540898714652634</v>
+        <v>0.615570301973216</v>
       </c>
     </row>
     <row r="44">
@@ -1299,16 +1299,16 @@
         <v>16</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.0521917982384489</v>
+        <v>-0.0528908827597301</v>
       </c>
       <c r="D44" t="n">
-        <v>-0.751238866659759</v>
+        <v>-0.763437001503801</v>
       </c>
       <c r="E44" t="n">
-        <v>0.452920807250981</v>
+        <v>0.445622448787831</v>
       </c>
       <c r="F44" t="n">
-        <v>0.751880675854233</v>
+        <v>0.728755774886901</v>
       </c>
     </row>
     <row r="45">
@@ -1319,16 +1319,16 @@
         <v>17</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.109832299275072</v>
+        <v>0.0170929005462158</v>
       </c>
       <c r="D45" t="n">
-        <v>-1.58090533024126</v>
+        <v>0.246722158132349</v>
       </c>
       <c r="E45" t="n">
-        <v>0.114636651070569</v>
+        <v>0.80524127343169</v>
       </c>
       <c r="F45" t="n">
-        <v>0.540898714652634</v>
+        <v>0.885765400774859</v>
       </c>
     </row>
     <row r="46">
@@ -1339,16 +1339,16 @@
         <v>7</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.0824913161283707</v>
+        <v>-0.0892040134700857</v>
       </c>
       <c r="D46" t="n">
-        <v>-1.07908274152652</v>
+        <v>-1.1564569324821</v>
       </c>
       <c r="E46" t="n">
-        <v>0.281157166697679</v>
+        <v>0.248137884170261</v>
       </c>
       <c r="F46" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="47">
@@ -1359,16 +1359,16 @@
         <v>8</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0380302779130285</v>
+        <v>0.0523538404814075</v>
       </c>
       <c r="D47" t="n">
-        <v>0.49748044372991</v>
+        <v>0.678724638181096</v>
       </c>
       <c r="E47" t="n">
-        <v>0.619105171121224</v>
+        <v>0.497678323411785</v>
       </c>
       <c r="F47" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="48">
@@ -1379,16 +1379,16 @@
         <v>9</v>
       </c>
       <c r="C48" t="n">
-        <v>-0.0479359899891019</v>
+        <v>-0.0521669247807174</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.62705872475997</v>
+        <v>-0.676301429297952</v>
       </c>
       <c r="E48" t="n">
-        <v>0.530954309851595</v>
+        <v>0.499213728810329</v>
       </c>
       <c r="F48" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="49">
@@ -1399,16 +1399,16 @@
         <v>10</v>
       </c>
       <c r="C49" t="n">
-        <v>0.0664936558031391</v>
+        <v>0.0597525285068298</v>
       </c>
       <c r="D49" t="n">
-        <v>0.869814663721854</v>
+        <v>0.77464256524994</v>
       </c>
       <c r="E49" t="n">
-        <v>0.384888103779534</v>
+        <v>0.438977626701592</v>
       </c>
       <c r="F49" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="50">
@@ -1419,16 +1419,16 @@
         <v>11</v>
       </c>
       <c r="C50" t="n">
-        <v>-0.101254381201523</v>
+        <v>0.000790828480422799</v>
       </c>
       <c r="D50" t="n">
-        <v>-1.32452554264597</v>
+        <v>0.0102524431694536</v>
       </c>
       <c r="E50" t="n">
-        <v>0.186033723986584</v>
+        <v>0.991824643102634</v>
       </c>
       <c r="F50" t="n">
-        <v>0.817821017702153</v>
+        <v>0.991824643102634</v>
       </c>
     </row>
     <row r="51">
@@ -1439,16 +1439,16 @@
         <v>12</v>
       </c>
       <c r="C51" t="n">
-        <v>0.055700183525113</v>
+        <v>0.0563406617206116</v>
       </c>
       <c r="D51" t="n">
-        <v>0.728623442596978</v>
+        <v>0.730410508371124</v>
       </c>
       <c r="E51" t="n">
-        <v>0.466629583619688</v>
+        <v>0.465537979376877</v>
       </c>
       <c r="F51" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="52">
@@ -1459,16 +1459,16 @@
         <v>13</v>
       </c>
       <c r="C52" t="n">
-        <v>0.0205292519744194</v>
+        <v>-0.0254205461990204</v>
       </c>
       <c r="D52" t="n">
-        <v>0.268546588195678</v>
+        <v>-0.329556549484144</v>
       </c>
       <c r="E52" t="n">
-        <v>0.788407708561996</v>
+        <v>0.741895903803947</v>
       </c>
       <c r="F52" t="n">
-        <v>0.817821017702153</v>
+        <v>0.906761660204824</v>
       </c>
     </row>
     <row r="53">
@@ -1479,16 +1479,16 @@
         <v>14</v>
       </c>
       <c r="C53" t="n">
-        <v>-0.0248568094299941</v>
+        <v>-0.0954773365369553</v>
       </c>
       <c r="D53" t="n">
-        <v>-0.325156093079903</v>
+        <v>-1.23778542509318</v>
       </c>
       <c r="E53" t="n">
-        <v>0.745221450791998</v>
+        <v>0.216472628996663</v>
       </c>
       <c r="F53" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="54">
@@ -1499,16 +1499,16 @@
         <v>15</v>
       </c>
       <c r="C54" t="n">
-        <v>-0.0176199755287301</v>
+        <v>-0.00592999795042485</v>
       </c>
       <c r="D54" t="n">
-        <v>-0.230489855072551</v>
+        <v>-0.0768775638292684</v>
       </c>
       <c r="E54" t="n">
-        <v>0.817821017702153</v>
+        <v>0.93875678641436</v>
       </c>
       <c r="F54" t="n">
-        <v>0.817821017702153</v>
+        <v>0.991824643102634</v>
       </c>
     </row>
     <row r="55">
@@ -1519,16 +1519,16 @@
         <v>16</v>
       </c>
       <c r="C55" t="n">
-        <v>0.0327548964787683</v>
+        <v>0.0303885736072217</v>
       </c>
       <c r="D55" t="n">
-        <v>0.428472294413673</v>
+        <v>0.393962953562611</v>
       </c>
       <c r="E55" t="n">
-        <v>0.668522347161275</v>
+        <v>0.693804135936233</v>
       </c>
       <c r="F55" t="n">
-        <v>0.817821017702153</v>
+        <v>0.906761660204824</v>
       </c>
     </row>
     <row r="56">
@@ -1539,16 +1539,16 @@
         <v>17</v>
       </c>
       <c r="C56" t="n">
-        <v>-0.0398879738502371</v>
+        <v>-0.0518948045893386</v>
       </c>
       <c r="D56" t="n">
-        <v>-0.521781275852969</v>
+        <v>-0.672773614017601</v>
       </c>
       <c r="E56" t="n">
-        <v>0.602091909135782</v>
+        <v>0.50145354655015</v>
       </c>
       <c r="F56" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="57">
@@ -1559,16 +1559,16 @@
         <v>7</v>
       </c>
       <c r="C57" t="n">
-        <v>0.00304088247626602</v>
+        <v>0.0142558917668867</v>
       </c>
       <c r="D57" t="n">
-        <v>0.0397643254502858</v>
+        <v>0.184729178423445</v>
       </c>
       <c r="E57" t="n">
-        <v>0.968299516204039</v>
+        <v>0.853528754311322</v>
       </c>
       <c r="F57" t="n">
-        <v>0.968299516204039</v>
+        <v>0.934619895185784</v>
       </c>
     </row>
     <row r="58">
@@ -1579,16 +1579,16 @@
         <v>8</v>
       </c>
       <c r="C58" t="n">
-        <v>0.0360039187658029</v>
+        <v>0.0297015893098577</v>
       </c>
       <c r="D58" t="n">
-        <v>0.470807916604204</v>
+        <v>0.384875971338749</v>
       </c>
       <c r="E58" t="n">
-        <v>0.638017204278547</v>
+        <v>0.700520042093063</v>
       </c>
       <c r="F58" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="59">
@@ -1599,16 +1599,16 @@
         <v>9</v>
       </c>
       <c r="C59" t="n">
-        <v>0.0860972300441796</v>
+        <v>-0.0432250552688277</v>
       </c>
       <c r="D59" t="n">
-        <v>1.12585682036907</v>
+        <v>-0.560114307662309</v>
       </c>
       <c r="E59" t="n">
-        <v>0.260855560091162</v>
+        <v>0.575693828960525</v>
       </c>
       <c r="F59" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="60">
@@ -1619,16 +1619,16 @@
         <v>10</v>
       </c>
       <c r="C60" t="n">
-        <v>-0.0490462702728194</v>
+        <v>-0.0477342484394711</v>
       </c>
       <c r="D60" t="n">
-        <v>-0.641357194325341</v>
+        <v>-0.618544854371451</v>
       </c>
       <c r="E60" t="n">
-        <v>0.521633130972589</v>
+        <v>0.536544511799657</v>
       </c>
       <c r="F60" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="61">
@@ -1639,16 +1639,16 @@
         <v>11</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.0471659631236178</v>
+        <v>-0.00633440916779664</v>
       </c>
       <c r="D61" t="n">
-        <v>-0.616769218298341</v>
+        <v>-0.0820818662556778</v>
       </c>
       <c r="E61" t="n">
-        <v>0.53771412692509</v>
+        <v>0.934619895185784</v>
       </c>
       <c r="F61" t="n">
-        <v>0.779798805229336</v>
+        <v>0.934619895185784</v>
       </c>
     </row>
     <row r="62">
@@ -1659,16 +1659,16 @@
         <v>12</v>
       </c>
       <c r="C62" t="n">
-        <v>-0.0397068520838941</v>
+        <v>-0.0386649949662801</v>
       </c>
       <c r="D62" t="n">
-        <v>-0.519229599037026</v>
+        <v>-0.501024619901937</v>
       </c>
       <c r="E62" t="n">
-        <v>0.603868400994964</v>
+        <v>0.616610765504908</v>
       </c>
       <c r="F62" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="63">
@@ -1679,16 +1679,16 @@
         <v>13</v>
       </c>
       <c r="C63" t="n">
-        <v>0.0254845341326823</v>
+        <v>0.0791082237904604</v>
       </c>
       <c r="D63" t="n">
-        <v>0.333250402509882</v>
+        <v>1.0250917603972</v>
       </c>
       <c r="E63" t="n">
-        <v>0.739108082512013</v>
+        <v>0.305897554077598</v>
       </c>
       <c r="F63" t="n">
-        <v>0.813018890763214</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="64">
@@ -1699,16 +1699,16 @@
         <v>14</v>
       </c>
       <c r="C64" t="n">
-        <v>0.0768162107058077</v>
+        <v>-0.0372697371117135</v>
       </c>
       <c r="D64" t="n">
-        <v>1.00449288198544</v>
+        <v>-0.482944738167591</v>
       </c>
       <c r="E64" t="n">
-        <v>0.315707331909155</v>
+        <v>0.629381331979864</v>
       </c>
       <c r="F64" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="65">
@@ -1719,16 +1719,16 @@
         <v>15</v>
       </c>
       <c r="C65" t="n">
-        <v>0.0648812589099049</v>
+        <v>0.0684061892253046</v>
       </c>
       <c r="D65" t="n">
-        <v>0.848424598797949</v>
+        <v>0.886413795875003</v>
       </c>
       <c r="E65" t="n">
-        <v>0.39667468693565</v>
+        <v>0.375891207982067</v>
       </c>
       <c r="F65" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="66">
@@ -1739,16 +1739,16 @@
         <v>16</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.064404183583889</v>
+        <v>-0.065414268217409</v>
       </c>
       <c r="D66" t="n">
-        <v>-0.842186087880128</v>
+        <v>-0.847644203713804</v>
       </c>
       <c r="E66" t="n">
-        <v>0.400153048945474</v>
+        <v>0.397108801556765</v>
       </c>
       <c r="F66" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="67">
@@ -1759,16 +1759,16 @@
         <v>17</v>
       </c>
       <c r="C67" t="n">
-        <v>-0.0539289181325395</v>
+        <v>0.0798099318237034</v>
       </c>
       <c r="D67" t="n">
-        <v>-0.70520550154156</v>
+        <v>1.03418455870079</v>
       </c>
       <c r="E67" t="n">
-        <v>0.481065066356249</v>
+        <v>0.301632515348916</v>
       </c>
       <c r="F67" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="68">
@@ -1779,16 +1779,16 @@
         <v>7</v>
       </c>
       <c r="C68" t="n">
-        <v>-0.108265601753358</v>
+        <v>-0.106421377337123</v>
       </c>
       <c r="D68" t="n">
-        <v>-1.41574317876234</v>
+        <v>-1.3790181578007</v>
       </c>
       <c r="E68" t="n">
-        <v>0.157576284908472</v>
+        <v>0.168607688667761</v>
       </c>
       <c r="F68" t="n">
-        <v>0.346667826798639</v>
+        <v>0.393587088958638</v>
       </c>
     </row>
     <row r="69">
@@ -1799,16 +1799,16 @@
         <v>8</v>
       </c>
       <c r="C69" t="n">
-        <v>0.00298907690208906</v>
+        <v>0.0734052026251266</v>
       </c>
       <c r="D69" t="n">
-        <v>0.0390868860136125</v>
+        <v>0.951191478911423</v>
       </c>
       <c r="E69" t="n">
-        <v>0.968839299111306</v>
+        <v>0.34204275839881</v>
       </c>
       <c r="F69" t="n">
-        <v>0.968839299111306</v>
+        <v>0.537495763198129</v>
       </c>
     </row>
     <row r="70">
@@ -1819,16 +1819,16 @@
         <v>9</v>
       </c>
       <c r="C70" t="n">
-        <v>-0.121601165478601</v>
+        <v>-0.127483797434826</v>
       </c>
       <c r="D70" t="n">
-        <v>-1.59012666782264</v>
+        <v>-1.65194696673678</v>
       </c>
       <c r="E70" t="n">
-        <v>0.112542877714915</v>
+        <v>0.0992770645365219</v>
       </c>
       <c r="F70" t="n">
-        <v>0.309492913716018</v>
+        <v>0.377330563669873</v>
       </c>
     </row>
     <row r="71">
@@ -1839,16 +1839,16 @@
         <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>0.124656181263922</v>
+        <v>0.103899686123902</v>
       </c>
       <c r="D71" t="n">
-        <v>1.63007580853802</v>
+        <v>1.34634184728479</v>
       </c>
       <c r="E71" t="n">
-        <v>0.103819433855277</v>
+        <v>0.178903222253926</v>
       </c>
       <c r="F71" t="n">
-        <v>0.309492913716018</v>
+        <v>0.393587088958638</v>
       </c>
     </row>
     <row r="72">
@@ -1859,16 +1859,16 @@
         <v>11</v>
       </c>
       <c r="C72" t="n">
-        <v>-0.0792580564314036</v>
+        <v>0.129300145174607</v>
       </c>
       <c r="D72" t="n">
-        <v>-1.03642385889422</v>
+        <v>1.67548337057511</v>
       </c>
       <c r="E72" t="n">
-        <v>0.300588282377239</v>
+        <v>0.0945680870997239</v>
       </c>
       <c r="F72" t="n">
-        <v>0.551078517691606</v>
+        <v>0.377330563669873</v>
       </c>
     </row>
     <row r="73">
@@ -1879,16 +1879,16 @@
         <v>12</v>
       </c>
       <c r="C73" t="n">
-        <v>-0.0206997662422272</v>
+        <v>-0.0189102489858781</v>
       </c>
       <c r="D73" t="n">
-        <v>-0.27068202997818</v>
+        <v>-0.245040774443739</v>
       </c>
       <c r="E73" t="n">
-        <v>0.786765779684009</v>
+        <v>0.806542029502812</v>
       </c>
       <c r="F73" t="n">
-        <v>0.916027362498677</v>
+        <v>0.887196232453093</v>
       </c>
     </row>
     <row r="74">
@@ -1899,16 +1899,16 @@
         <v>13</v>
       </c>
       <c r="C74" t="n">
-        <v>0.162774717771661</v>
+        <v>-0.0104899559164335</v>
       </c>
       <c r="D74" t="n">
-        <v>2.12853568102989</v>
+        <v>-0.13592982956296</v>
       </c>
       <c r="E74" t="n">
-        <v>0.033861927042385</v>
+        <v>0.891940513699548</v>
       </c>
       <c r="F74" t="n">
-        <v>0.309492913716018</v>
+        <v>0.891940513699548</v>
       </c>
     </row>
     <row r="75">
@@ -1919,16 +1919,16 @@
         <v>14</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.016158801021707</v>
+        <v>-0.0807295555999448</v>
       </c>
       <c r="D75" t="n">
-        <v>-0.211301761159334</v>
+        <v>-1.046101129577</v>
       </c>
       <c r="E75" t="n">
-        <v>0.83275214772607</v>
+        <v>0.29610339140055</v>
       </c>
       <c r="F75" t="n">
-        <v>0.916027362498677</v>
+        <v>0.537495763198129</v>
       </c>
     </row>
     <row r="76">
@@ -1939,16 +1939,16 @@
         <v>15</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.0540594463270421</v>
+        <v>-0.0510296506770713</v>
       </c>
       <c r="D76" t="n">
-        <v>-0.70691236316714</v>
+        <v>-0.661246984682281</v>
       </c>
       <c r="E76" t="n">
-        <v>0.480004729514559</v>
+        <v>0.508808900092943</v>
       </c>
       <c r="F76" t="n">
-        <v>0.660006503082519</v>
+        <v>0.623107021641293</v>
       </c>
     </row>
     <row r="77">
@@ -1959,16 +1959,16 @@
         <v>16</v>
       </c>
       <c r="C77" t="n">
-        <v>0.0541412747986264</v>
+        <v>0.0509085248848264</v>
       </c>
       <c r="D77" t="n">
-        <v>0.707982399250604</v>
+        <v>0.659677425341261</v>
       </c>
       <c r="E77" t="n">
-        <v>0.47934065424041</v>
+        <v>0.509814835888331</v>
       </c>
       <c r="F77" t="n">
-        <v>0.660006503082519</v>
+        <v>0.623107021641293</v>
       </c>
     </row>
     <row r="78">
@@ -1979,16 +1979,16 @@
         <v>17</v>
       </c>
       <c r="C78" t="n">
-        <v>-0.126425571546606</v>
+        <v>-0.126129705694016</v>
       </c>
       <c r="D78" t="n">
-        <v>-1.65321337192574</v>
+        <v>-1.63440051935347</v>
       </c>
       <c r="E78" t="n">
-        <v>0.0990190003951576</v>
+        <v>0.102908335546329</v>
       </c>
       <c r="F78" t="n">
-        <v>0.309492913716018</v>
+        <v>0.377330563669873</v>
       </c>
     </row>
     <row r="79">
@@ -1999,16 +1999,16 @@
         <v>7</v>
       </c>
       <c r="C79" t="n">
-        <v>0.0855321986046367</v>
+        <v>0.103459905236972</v>
       </c>
       <c r="D79" t="n">
-        <v>0.837425477701765</v>
+        <v>1.01503264438571</v>
       </c>
       <c r="E79" t="n">
-        <v>0.402819725128278</v>
+        <v>0.310662378006296</v>
       </c>
       <c r="F79" t="n">
-        <v>0.65950051515095</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="80">
@@ -2019,16 +2019,16 @@
         <v>8</v>
       </c>
       <c r="C80" t="n">
-        <v>-0.00202635914722561</v>
+        <v>-0.0226522511715498</v>
       </c>
       <c r="D80" t="n">
-        <v>-0.0198396019808236</v>
+        <v>-0.222238502493145</v>
       </c>
       <c r="E80" t="n">
-        <v>0.984180550172677</v>
+        <v>0.824233983060949</v>
       </c>
       <c r="F80" t="n">
-        <v>0.984180550172677</v>
+        <v>0.944301968554532</v>
       </c>
     </row>
     <row r="81">
@@ -2039,16 +2039,16 @@
         <v>9</v>
       </c>
       <c r="C81" t="n">
-        <v>0.134033220033281</v>
+        <v>0.00894186951188972</v>
       </c>
       <c r="D81" t="n">
-        <v>1.31228747939834</v>
+        <v>0.0877276026458397</v>
       </c>
       <c r="E81" t="n">
-        <v>0.190124840249583</v>
+        <v>0.930134114993142</v>
       </c>
       <c r="F81" t="n">
-        <v>0.65950051515095</v>
+        <v>0.944301968554532</v>
       </c>
     </row>
     <row r="82">
@@ -2059,16 +2059,16 @@
         <v>10</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.115539926075959</v>
+        <v>-0.107486776946301</v>
       </c>
       <c r="D82" t="n">
-        <v>-1.13122402283882</v>
+        <v>-1.05453979674932</v>
       </c>
       <c r="E82" t="n">
-        <v>0.258592783785286</v>
+        <v>0.292229389917742</v>
       </c>
       <c r="F82" t="n">
-        <v>0.65950051515095</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="83">
@@ -2079,16 +2079,16 @@
         <v>11</v>
       </c>
       <c r="C83" t="n">
-        <v>0.0540884180779053</v>
+        <v>-0.00712523764821944</v>
       </c>
       <c r="D83" t="n">
-        <v>0.529566877573134</v>
+        <v>-0.0699048466686998</v>
       </c>
       <c r="E83" t="n">
-        <v>0.596686197717115</v>
+        <v>0.944301968554532</v>
       </c>
       <c r="F83" t="n">
-        <v>0.820443521861032</v>
+        <v>0.944301968554532</v>
       </c>
     </row>
     <row r="84">
@@ -2099,16 +2099,16 @@
         <v>12</v>
       </c>
       <c r="C84" t="n">
-        <v>-0.0954070356090071</v>
+        <v>-0.0950056566868917</v>
       </c>
       <c r="D84" t="n">
-        <v>-0.934107665585612</v>
+        <v>-0.932089032148414</v>
       </c>
       <c r="E84" t="n">
-        <v>0.35077381883406</v>
+        <v>0.35181477304789</v>
       </c>
       <c r="F84" t="n">
-        <v>0.65950051515095</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="85">
@@ -2119,16 +2119,16 @@
         <v>13</v>
       </c>
       <c r="C85" t="n">
-        <v>0.00495528215826297</v>
+        <v>0.104528769989481</v>
       </c>
       <c r="D85" t="n">
-        <v>0.0485159927632849</v>
+        <v>1.02551914747832</v>
       </c>
       <c r="E85" t="n">
-        <v>0.961327597329494</v>
+        <v>0.305696191005939</v>
       </c>
       <c r="F85" t="n">
-        <v>0.984180550172677</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="86">
@@ -2139,16 +2139,16 @@
         <v>14</v>
       </c>
       <c r="C86" t="n">
-        <v>0.101673020135802</v>
+        <v>0.0582075994252418</v>
       </c>
       <c r="D86" t="n">
-        <v>0.995456434484654</v>
+        <v>0.571067733269423</v>
       </c>
       <c r="E86" t="n">
-        <v>0.320075462248847</v>
+        <v>0.56825275598031</v>
       </c>
       <c r="F86" t="n">
-        <v>0.65950051515095</v>
+        <v>0.781347539472926</v>
       </c>
     </row>
     <row r="87">
@@ -2159,16 +2159,16 @@
         <v>15</v>
       </c>
       <c r="C87" t="n">
-        <v>0.0825012344386349</v>
+        <v>0.0743361871757295</v>
       </c>
       <c r="D87" t="n">
-        <v>0.807750026163993</v>
+        <v>0.729303361236479</v>
       </c>
       <c r="E87" t="n">
-        <v>0.41968214600515</v>
+        <v>0.466214096888846</v>
       </c>
       <c r="F87" t="n">
-        <v>0.65950051515095</v>
+        <v>0.732622152253901</v>
       </c>
     </row>
     <row r="88">
@@ -2179,16 +2179,16 @@
         <v>16</v>
       </c>
       <c r="C88" t="n">
-        <v>-0.0971590800626574</v>
+        <v>-0.0958028418246307</v>
       </c>
       <c r="D88" t="n">
-        <v>-0.951261517438933</v>
+        <v>-0.93991011932775</v>
       </c>
       <c r="E88" t="n">
-        <v>0.342007253225118</v>
+        <v>0.347792576376125</v>
       </c>
       <c r="F88" t="n">
-        <v>0.65950051515095</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="89">
@@ -2199,16 +2199,16 @@
         <v>17</v>
       </c>
       <c r="C89" t="n">
-        <v>-0.0140409442823025</v>
+        <v>0.131704736413042</v>
       </c>
       <c r="D89" t="n">
-        <v>-0.137471556499351</v>
+        <v>1.29213927437157</v>
       </c>
       <c r="E89" t="n">
-        <v>0.890722570103284</v>
+        <v>0.19700451886975</v>
       </c>
       <c r="F89" t="n">
-        <v>0.984180550172677</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="90">
@@ -2219,16 +2219,16 @@
         <v>7</v>
       </c>
       <c r="C90" t="n">
-        <v>-0.111306484229624</v>
+        <v>-0.12067726910401</v>
       </c>
       <c r="D90" t="n">
-        <v>-1.09445937065408</v>
+        <v>-1.18992956091244</v>
       </c>
       <c r="E90" t="n">
-        <v>0.274367664727275</v>
+        <v>0.234732176589991</v>
       </c>
       <c r="F90" t="n">
-        <v>0.503007385333338</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
     <row r="91">
@@ -2239,16 +2239,16 @@
         <v>8</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.0330148418637138</v>
+        <v>0.0437036133152689</v>
       </c>
       <c r="D91" t="n">
-        <v>-0.324629811987067</v>
+        <v>0.430936346079421</v>
       </c>
       <c r="E91" t="n">
-        <v>0.745619496610592</v>
+        <v>0.666731095715551</v>
       </c>
       <c r="F91" t="n">
-        <v>0.827741812715881</v>
+        <v>0.735326473915939</v>
       </c>
     </row>
     <row r="92">
@@ -2259,16 +2259,16 @@
         <v>9</v>
       </c>
       <c r="C92" t="n">
-        <v>-0.20769839552278</v>
+        <v>-0.0842587421659985</v>
       </c>
       <c r="D92" t="n">
-        <v>-2.0422660622428</v>
+        <v>-0.830827286804171</v>
       </c>
       <c r="E92" t="n">
-        <v>0.0417360760492035</v>
+        <v>0.406533351975047</v>
       </c>
       <c r="F92" t="n">
-        <v>0.459096836541238</v>
+        <v>0.55898335896569</v>
       </c>
     </row>
     <row r="93">
@@ -2279,16 +2279,16 @@
         <v>10</v>
       </c>
       <c r="C93" t="n">
-        <v>0.173702451536742</v>
+        <v>0.151633934563373</v>
       </c>
       <c r="D93" t="n">
-        <v>1.70798922547745</v>
+        <v>1.49517554145933</v>
       </c>
       <c r="E93" t="n">
-        <v>0.0883617586478161</v>
+        <v>0.135603851364239</v>
       </c>
       <c r="F93" t="n">
-        <v>0.485989672562989</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
     <row r="94">
@@ -2299,16 +2299,16 @@
         <v>11</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.0320920933077857</v>
+        <v>0.135634554342404</v>
       </c>
       <c r="D94" t="n">
-        <v>-0.315556568763342</v>
+        <v>1.33741479975079</v>
       </c>
       <c r="E94" t="n">
-        <v>0.752492557014437</v>
+        <v>0.181795908284388</v>
       </c>
       <c r="F94" t="n">
-        <v>0.827741812715881</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
     <row r="95">
@@ -2319,16 +2319,16 @@
         <v>12</v>
       </c>
       <c r="C95" t="n">
-        <v>0.0190070858416669</v>
+        <v>0.019754745980402</v>
       </c>
       <c r="D95" t="n">
-        <v>0.186893722789084</v>
+        <v>0.194790256565522</v>
       </c>
       <c r="E95" t="n">
-        <v>0.851832312336532</v>
+        <v>0.845649363699252</v>
       </c>
       <c r="F95" t="n">
-        <v>0.851832312336532</v>
+        <v>0.845649363699252</v>
       </c>
     </row>
     <row r="96">
@@ -2339,16 +2339,16 @@
         <v>13</v>
       </c>
       <c r="C96" t="n">
-        <v>0.137290183638979</v>
+        <v>-0.0895981797068938</v>
       </c>
       <c r="D96" t="n">
-        <v>1.34995305100571</v>
+        <v>-0.883476427903651</v>
       </c>
       <c r="E96" t="n">
-        <v>0.177742871318337</v>
+        <v>0.377473731733483</v>
       </c>
       <c r="F96" t="n">
-        <v>0.503007385333338</v>
+        <v>0.55898335896569</v>
       </c>
     </row>
     <row r="97">
@@ -2359,16 +2359,16 @@
         <v>14</v>
       </c>
       <c r="C97" t="n">
-        <v>-0.0929750117275147</v>
+        <v>-0.0434598184882313</v>
       </c>
       <c r="D97" t="n">
-        <v>-0.914208848892642</v>
+        <v>-0.428532424664532</v>
       </c>
       <c r="E97" t="n">
-        <v>0.361120643427405</v>
+        <v>0.668478612650854</v>
       </c>
       <c r="F97" t="n">
-        <v>0.567475296814493</v>
+        <v>0.735326473915939</v>
       </c>
     </row>
     <row r="98">
@@ -2379,16 +2379,16 @@
         <v>15</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.118940705236947</v>
+        <v>-0.119435839902376</v>
       </c>
       <c r="D98" t="n">
-        <v>-1.16952548002712</v>
+        <v>-1.17768853726506</v>
       </c>
       <c r="E98" t="n">
-        <v>0.242841351016825</v>
+        <v>0.239573706301444</v>
       </c>
       <c r="F98" t="n">
-        <v>0.503007385333338</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
     <row r="99">
@@ -2399,16 +2399,16 @@
         <v>16</v>
       </c>
       <c r="C99" t="n">
-        <v>0.118545458382515</v>
+        <v>0.116322793102235</v>
       </c>
       <c r="D99" t="n">
-        <v>1.16563907909955</v>
+        <v>1.14699256245974</v>
       </c>
       <c r="E99" t="n">
-        <v>0.244408064073736</v>
+        <v>0.25202398402972</v>
       </c>
       <c r="F99" t="n">
-        <v>0.503007385333338</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
     <row r="100">
@@ -2419,16 +2419,16 @@
         <v>17</v>
       </c>
       <c r="C100" t="n">
-        <v>-0.0724966534140664</v>
+        <v>-0.205939637517719</v>
       </c>
       <c r="D100" t="n">
-        <v>-0.7128483324152</v>
+        <v>-2.03065303238441</v>
       </c>
       <c r="E100" t="n">
-        <v>0.476327162749557</v>
+        <v>0.0429064644520612</v>
       </c>
       <c r="F100" t="n">
-        <v>0.654949848780641</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
   </sheetData>
@@ -2473,7 +2473,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0761757033103153</v>
+        <v>0.0697935914744919</v>
       </c>
     </row>
     <row r="3">
@@ -2484,13 +2484,13 @@
         <v>11</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.309492913716018</v>
+        <v>0.377330563669873</v>
       </c>
     </row>
     <row r="4">
@@ -2507,7 +2507,7 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.459096836541238</v>
+        <v>0.462043970721153</v>
       </c>
     </row>
     <row r="5">
@@ -2518,13 +2518,13 @@
         <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.152453458389753</v>
+        <v>0.615570301973216</v>
       </c>
     </row>
     <row r="6">
@@ -2541,7 +2541,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0.817821017702153</v>
+        <v>0.787998430293093</v>
       </c>
     </row>
     <row r="7">
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.779798805229336</v>
+        <v>0.856191162558189</v>
       </c>
     </row>
     <row r="8">
@@ -2569,13 +2569,13 @@
         <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0.224478847415378</v>
+        <v>0.236962350301216</v>
       </c>
     </row>
     <row r="9">
@@ -2592,7 +2592,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0.65950051515095</v>
+        <v>0.644993750587798</v>
       </c>
     </row>
     <row r="10">
@@ -2609,7 +2609,7 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>0.950327173765851</v>
+        <v>0.935525204626051</v>
       </c>
     </row>
   </sheetData>

</xml_diff>